<commit_message>
Test harness: HAVS and Projects checks follow the current screens
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012KhfNvBEbifMJmPdX7yZfp
</commit_message>
<xml_diff>
--- a/tools/test-harness/shots/app-test.xlsx
+++ b/tools/test-harness/shots/app-test.xlsx
@@ -1333,13 +1333,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16FBDBD8-2E48-4072-97A4-9E2EBA3B6CA1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3FC0D766-ABE1-4BB3-BD71-04D54FDF0085}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{61DB5F14-4FFD-44FD-935C-EA18711BD00F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3A62A3D-7A34-4DFF-862E-06EF6AF71FF4}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B91AC96-3FFA-416C-95B1-1012DCBE07AB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CA689BE-A36A-4788-97FF-0F37B3821A9D}"/>
 </file>
</xml_diff>